<commit_message>
fix: refine function to calculate the structure size
</commit_message>
<xml_diff>
--- a/data/all_component_manual_check.xlsx
+++ b/data/all_component_manual_check.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0248A341-C234-114C-9B20-2EFA130D717D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA55A71-B895-A64D-9C30-6414F45668A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31960" yWindow="7340" windowWidth="26760" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="31960" yWindow="4580" windowWidth="26760" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="344">
   <si>
     <t>GO_Name</t>
   </si>
@@ -1053,6 +1053,9 @@
   </si>
   <si>
     <t>Frequency</t>
+  </si>
+  <si>
+    <t>all the living material in a cell, not including the nucleus</t>
   </si>
 </sst>
 </file>
@@ -1551,16 +1554,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C318"/>
+  <dimension ref="A1:D318"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.33203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="45.33203125" style="2" customWidth="1"/>
     <col min="2" max="2" width="10" style="5" customWidth="1"/>
     <col min="3" max="3" width="43.83203125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1570,8 +1572,11 @@
       <c r="C1" s="6" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="D1" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1582,15 +1587,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="5">
         <v>11432</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+      <c r="D3" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1601,7 +1609,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -1609,7 +1617,7 @@
         <v>4849</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -1620,7 +1628,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1628,7 +1636,7 @@
         <v>2395</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
         <v>7</v>
       </c>
@@ -1639,7 +1647,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>8</v>
       </c>
@@ -1650,7 +1658,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1658,7 +1666,7 @@
         <v>1364</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -1669,7 +1677,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -1677,7 +1685,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>12</v>
       </c>
@@ -1688,7 +1696,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -1699,7 +1707,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="8" t="s">
         <v>14</v>
       </c>
@@ -1710,7 +1718,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
@@ -1721,7 +1729,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -1729,7 +1737,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
@@ -1740,7 +1748,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
@@ -1748,7 +1756,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="9" t="s">
         <v>19</v>
       </c>
@@ -1756,7 +1764,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -1767,7 +1775,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -1775,7 +1783,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="9" t="s">
         <v>22</v>
       </c>
@@ -1783,7 +1791,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
@@ -1791,7 +1799,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
@@ -1802,7 +1810,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
@@ -1810,7 +1818,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
         <v>26</v>
       </c>
@@ -1821,7 +1829,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
@@ -1832,7 +1840,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
@@ -1843,7 +1851,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
@@ -1851,7 +1859,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
@@ -1862,7 +1870,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
         <v>31</v>
       </c>
@@ -1884,7 +1892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>33</v>
       </c>
@@ -1906,7 +1914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>35</v>
       </c>
@@ -1914,7 +1922,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>36</v>
       </c>
@@ -1925,7 +1933,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
@@ -1936,7 +1944,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
@@ -1944,7 +1952,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
@@ -1952,7 +1960,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>40</v>
       </c>
@@ -1963,7 +1971,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>41</v>
       </c>
@@ -1982,7 +1990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>43</v>
       </c>
@@ -1990,7 +1998,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="8" t="s">
         <v>44</v>
       </c>
@@ -2001,7 +2009,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>45</v>
       </c>
@@ -2020,7 +2028,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>47</v>
       </c>
@@ -2028,7 +2036,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="11" t="s">
         <v>48</v>
       </c>
@@ -2039,7 +2047,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>49</v>
       </c>
@@ -2047,7 +2055,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="9" t="s">
         <v>50</v>
       </c>
@@ -2066,7 +2074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>52</v>
       </c>
@@ -2088,7 +2096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>54</v>
       </c>
@@ -2099,7 +2107,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="9" t="s">
         <v>55</v>
       </c>
@@ -2107,7 +2115,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="13" t="s">
         <v>56</v>
       </c>
@@ -2115,7 +2123,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>57</v>
       </c>
@@ -2123,7 +2131,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
         <v>58</v>
       </c>
@@ -2131,7 +2139,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>59</v>
       </c>
@@ -2139,7 +2147,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="9" t="s">
         <v>60</v>
       </c>
@@ -2158,7 +2166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="11" t="s">
         <v>62</v>
       </c>
@@ -2169,7 +2177,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>63</v>
       </c>
@@ -2177,7 +2185,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="15" t="s">
         <v>64</v>
       </c>
@@ -2188,7 +2196,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>65</v>
       </c>
@@ -2196,7 +2204,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>66</v>
       </c>
@@ -2207,7 +2215,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>67</v>
       </c>
@@ -2215,7 +2223,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>68</v>
       </c>
@@ -2226,7 +2234,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>69</v>
       </c>
@@ -2234,7 +2242,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>70</v>
       </c>
@@ -2264,7 +2272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>73</v>
       </c>
@@ -2272,7 +2280,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>74</v>
       </c>
@@ -2280,7 +2288,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>75</v>
       </c>
@@ -2288,7 +2296,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>76</v>
       </c>
@@ -2296,7 +2304,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>77</v>
       </c>
@@ -2318,7 +2326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>79</v>
       </c>
@@ -2326,7 +2334,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="9" t="s">
         <v>80</v>
       </c>
@@ -2334,7 +2342,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>81</v>
       </c>
@@ -2342,7 +2350,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>82</v>
       </c>
@@ -2350,7 +2358,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>83</v>
       </c>
@@ -2361,7 +2369,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>84</v>
       </c>
@@ -2369,7 +2377,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>85</v>
       </c>
@@ -2377,7 +2385,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="22" t="s">
         <v>86</v>
       </c>
@@ -2388,7 +2396,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="22" t="s">
         <v>87</v>
       </c>
@@ -2399,7 +2407,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>88</v>
       </c>
@@ -2407,7 +2415,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="16" t="s">
         <v>89</v>
       </c>
@@ -2418,7 +2426,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="9" t="s">
         <v>90</v>
       </c>
@@ -2437,7 +2445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>92</v>
       </c>
@@ -2445,7 +2453,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="94" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>93</v>
       </c>
@@ -2453,7 +2461,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="95" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>94</v>
       </c>
@@ -2461,7 +2469,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>95</v>
       </c>
@@ -2469,7 +2477,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>96</v>
       </c>
@@ -2480,7 +2488,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>97</v>
       </c>
@@ -2488,7 +2496,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="15" t="s">
         <v>98</v>
       </c>
@@ -2510,7 +2518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="9" t="s">
         <v>100</v>
       </c>
@@ -2521,7 +2529,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="15" t="s">
         <v>101</v>
       </c>
@@ -2532,7 +2540,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>102</v>
       </c>
@@ -2540,7 +2548,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>103</v>
       </c>
@@ -2562,7 +2570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>105</v>
       </c>
@@ -2573,7 +2581,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>106</v>
       </c>
@@ -2584,7 +2592,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="17" t="s">
         <v>107</v>
       </c>
@@ -2592,7 +2600,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="9" t="s">
         <v>108</v>
       </c>
@@ -2603,7 +2611,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="9" t="s">
         <v>109</v>
       </c>
@@ -2611,7 +2619,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="16" t="s">
         <v>110</v>
       </c>
@@ -2619,7 +2627,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="9" t="s">
         <v>111</v>
       </c>
@@ -2627,7 +2635,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="8" t="s">
         <v>112</v>
       </c>
@@ -2638,7 +2646,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>113</v>
       </c>
@@ -2646,7 +2654,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>114</v>
       </c>
@@ -2654,7 +2662,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="116" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>115</v>
       </c>
@@ -2662,7 +2670,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" s="16" t="s">
         <v>116</v>
       </c>
@@ -2670,7 +2678,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>117</v>
       </c>
@@ -2700,7 +2708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>120</v>
       </c>
@@ -2708,7 +2716,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>121</v>
       </c>
@@ -2716,7 +2724,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="9" t="s">
         <v>122</v>
       </c>
@@ -2724,7 +2732,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>123</v>
       </c>
@@ -2732,7 +2740,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>124</v>
       </c>
@@ -2740,7 +2748,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" s="9" t="s">
         <v>125</v>
       </c>
@@ -2759,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>127</v>
       </c>
@@ -2767,7 +2775,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>128</v>
       </c>
@@ -2775,7 +2783,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>129</v>
       </c>
@@ -2786,7 +2794,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>130</v>
       </c>
@@ -2794,7 +2802,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="132" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>131</v>
       </c>
@@ -2802,7 +2810,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="133" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" s="19" t="s">
         <v>132</v>
       </c>
@@ -2810,7 +2818,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="134" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>133</v>
       </c>
@@ -2818,7 +2826,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>134</v>
       </c>
@@ -2826,7 +2834,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" s="15" t="s">
         <v>135</v>
       </c>
@@ -2848,7 +2856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>137</v>
       </c>
@@ -2856,7 +2864,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="139" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>138</v>
       </c>
@@ -2864,7 +2872,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>139</v>
       </c>
@@ -2883,7 +2891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>141</v>
       </c>
@@ -2891,7 +2899,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="143" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" s="17" t="s">
         <v>142</v>
       </c>
@@ -2899,7 +2907,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="144" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A144" s="12" t="s">
         <v>143</v>
       </c>
@@ -2910,7 +2918,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A145" s="17" t="s">
         <v>144</v>
       </c>
@@ -2918,7 +2926,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>145</v>
       </c>
@@ -2940,7 +2948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A148" s="14" t="s">
         <v>147</v>
       </c>
@@ -2948,7 +2956,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="149" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A149" s="17" t="s">
         <v>148</v>
       </c>
@@ -2959,7 +2967,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>149</v>
       </c>
@@ -2970,7 +2978,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="151" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>150</v>
       </c>
@@ -2978,7 +2986,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="152" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>151</v>
       </c>
@@ -2986,7 +2994,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="153" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>152</v>
       </c>
@@ -2994,7 +3002,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="154" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>153</v>
       </c>
@@ -3002,7 +3010,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="155" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>154</v>
       </c>
@@ -3010,7 +3018,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="156" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>155</v>
       </c>
@@ -3018,7 +3026,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" s="13" t="s">
         <v>156</v>
       </c>
@@ -3029,7 +3037,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="158" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>157</v>
       </c>
@@ -3037,7 +3045,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" s="17" t="s">
         <v>158</v>
       </c>
@@ -3057,7 +3065,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>160</v>
       </c>
@@ -3065,7 +3073,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="162" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>161</v>
       </c>
@@ -3084,7 +3092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>163</v>
       </c>
@@ -3095,7 +3103,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>164</v>
       </c>
@@ -3106,7 +3114,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>165</v>
       </c>
@@ -3117,7 +3125,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" s="1" t="s">
         <v>166</v>
       </c>
@@ -3125,7 +3133,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A168" s="8" t="s">
         <v>167</v>
       </c>
@@ -3136,7 +3144,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="169" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
         <v>168</v>
       </c>
@@ -3144,7 +3152,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="170" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
         <v>169</v>
       </c>
@@ -3152,7 +3160,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="171" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
         <v>170</v>
       </c>
@@ -3163,7 +3171,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="172" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
         <v>171</v>
       </c>
@@ -3171,7 +3179,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="173" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
         <v>172</v>
       </c>
@@ -3179,7 +3187,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="174" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A174" s="9" t="s">
         <v>173</v>
       </c>
@@ -3190,7 +3198,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="175" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
         <v>174</v>
       </c>
@@ -3198,7 +3206,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" s="15" t="s">
         <v>175</v>
       </c>
@@ -3209,7 +3217,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
         <v>176</v>
       </c>
@@ -3220,7 +3228,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
         <v>177</v>
       </c>
@@ -3231,7 +3239,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
         <v>178</v>
       </c>
@@ -3242,7 +3250,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A180" s="9" t="s">
         <v>179</v>
       </c>
@@ -3253,7 +3261,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A181" s="9" t="s">
         <v>180</v>
       </c>
@@ -3264,7 +3272,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
         <v>181</v>
       </c>
@@ -3272,7 +3280,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A183" s="11" t="s">
         <v>182</v>
       </c>
@@ -3283,7 +3291,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="184" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
         <v>183</v>
       </c>
@@ -3291,7 +3299,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="s">
         <v>184</v>
       </c>
@@ -3299,7 +3307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="186" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="s">
         <v>185</v>
       </c>
@@ -3307,7 +3315,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="187" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="s">
         <v>186</v>
       </c>
@@ -3315,7 +3323,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="188" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
         <v>187</v>
       </c>
@@ -3323,7 +3331,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="s">
         <v>188</v>
       </c>
@@ -3334,7 +3342,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="s">
         <v>189</v>
       </c>
@@ -3364,7 +3372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
         <v>192</v>
       </c>
@@ -3372,7 +3380,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="194" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" s="11" t="s">
         <v>193</v>
       </c>
@@ -3383,7 +3391,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="195" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
         <v>194</v>
       </c>
@@ -3391,7 +3399,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A196" s="9" t="s">
         <v>195</v>
       </c>
@@ -3399,7 +3407,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="197" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
         <v>196</v>
       </c>
@@ -3407,7 +3415,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="198" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
         <v>197</v>
       </c>
@@ -3418,7 +3426,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="199" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
         <v>198</v>
       </c>
@@ -3429,7 +3437,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="200" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A200" s="9" t="s">
         <v>199</v>
       </c>
@@ -3440,7 +3448,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="201" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
         <v>200</v>
       </c>
@@ -3451,7 +3459,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="202" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="s">
         <v>201</v>
       </c>
@@ -3459,7 +3467,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="203" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A203" s="12" t="s">
         <v>202</v>
       </c>
@@ -3467,7 +3475,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="204" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="s">
         <v>203</v>
       </c>
@@ -3478,7 +3486,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="205" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A205" s="1" t="s">
         <v>204</v>
       </c>
@@ -3497,7 +3505,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
         <v>206</v>
       </c>
@@ -3505,7 +3513,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="208" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A208" s="1" t="s">
         <v>207</v>
       </c>
@@ -3513,7 +3521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="s">
         <v>208</v>
       </c>
@@ -3524,7 +3532,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="210" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" s="11" t="s">
         <v>209</v>
       </c>
@@ -3535,7 +3543,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="211" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
         <v>210</v>
       </c>
@@ -3546,7 +3554,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="212" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="s">
         <v>211</v>
       </c>
@@ -3554,7 +3562,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="213" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="s">
         <v>212</v>
       </c>
@@ -3565,7 +3573,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="214" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" s="9" t="s">
         <v>213</v>
       </c>
@@ -3584,7 +3592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="s">
         <v>215</v>
       </c>
@@ -3592,7 +3600,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="217" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
         <v>216</v>
       </c>
@@ -3614,7 +3622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
         <v>218</v>
       </c>
@@ -3622,7 +3630,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="220" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
         <v>219</v>
       </c>
@@ -3630,7 +3638,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="221" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="s">
         <v>220</v>
       </c>
@@ -3641,7 +3649,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="222" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" s="8" t="s">
         <v>221</v>
       </c>
@@ -3663,7 +3671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
         <v>223</v>
       </c>
@@ -3671,7 +3679,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="225" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
         <v>224</v>
       </c>
@@ -3679,7 +3687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="226" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
         <v>225</v>
       </c>
@@ -3701,7 +3709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
         <v>227</v>
       </c>
@@ -3720,7 +3728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
         <v>229</v>
       </c>
@@ -3731,7 +3739,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="231" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="s">
         <v>230</v>
       </c>
@@ -3739,7 +3747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
         <v>231</v>
       </c>
@@ -3747,7 +3755,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="233" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="s">
         <v>232</v>
       </c>
@@ -3766,7 +3774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
         <v>234</v>
       </c>
@@ -3774,7 +3782,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="236" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="s">
         <v>235</v>
       </c>
@@ -3782,7 +3790,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="237" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="s">
         <v>236</v>
       </c>
@@ -3790,7 +3798,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="238" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="s">
         <v>237</v>
       </c>
@@ -3801,7 +3809,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="239" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="s">
         <v>238</v>
       </c>
@@ -3812,7 +3820,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="240" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A240" s="14" t="s">
         <v>239</v>
       </c>
@@ -3831,7 +3839,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="s">
         <v>241</v>
       </c>
@@ -3839,7 +3847,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="243" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
         <v>242</v>
       </c>
@@ -3850,7 +3858,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="244" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A244" s="16" t="s">
         <v>243</v>
       </c>
@@ -3859,7 +3867,7 @@
       </c>
       <c r="C244" s="4"/>
     </row>
-    <row r="245" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
         <v>244</v>
       </c>
@@ -3867,7 +3875,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="246" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
         <v>245</v>
       </c>
@@ -3878,7 +3886,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="247" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A247" s="8" t="s">
         <v>246</v>
       </c>
@@ -3889,7 +3897,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="248" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="s">
         <v>247</v>
       </c>
@@ -3897,7 +3905,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="249" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A249" s="16" t="s">
         <v>248</v>
       </c>
@@ -3905,7 +3913,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="250" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A250" s="1" t="s">
         <v>249</v>
       </c>
@@ -3913,7 +3921,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A251" s="1" t="s">
         <v>250</v>
       </c>
@@ -3921,7 +3929,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="252" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A252" s="9" t="s">
         <v>251</v>
       </c>
@@ -3932,7 +3940,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="253" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A253" s="1" t="s">
         <v>252</v>
       </c>
@@ -3940,7 +3948,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="254" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A254" s="16" t="s">
         <v>253</v>
       </c>
@@ -3948,7 +3956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="255" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A255" s="1" t="s">
         <v>254</v>
       </c>
@@ -3956,7 +3964,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="256" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A256" s="1" t="s">
         <v>255</v>
       </c>
@@ -3978,7 +3986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A258" s="8" t="s">
         <v>257</v>
       </c>
@@ -3989,7 +3997,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="259" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A259" s="1" t="s">
         <v>258</v>
       </c>
@@ -3997,7 +4005,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="260" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A260" s="3" t="s">
         <v>259</v>
       </c>
@@ -4005,7 +4013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A261" s="3" t="s">
         <v>260</v>
       </c>
@@ -4013,7 +4021,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="262" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A262" s="15" t="s">
         <v>261</v>
       </c>
@@ -4024,7 +4032,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="263" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A263" s="3" t="s">
         <v>262</v>
       </c>
@@ -4032,7 +4040,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A264" s="3" t="s">
         <v>263</v>
       </c>
@@ -4043,7 +4051,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="265" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A265" s="3" t="s">
         <v>264</v>
       </c>
@@ -4051,7 +4059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="266" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A266" s="8" t="s">
         <v>265</v>
       </c>
@@ -4062,7 +4070,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="267" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A267" s="3" t="s">
         <v>266</v>
       </c>
@@ -4070,7 +4078,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="268" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A268" s="3" t="s">
         <v>267</v>
       </c>
@@ -4081,7 +4089,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="269" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A269" s="3" t="s">
         <v>268</v>
       </c>
@@ -4089,7 +4097,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="270" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A270" s="3" t="s">
         <v>269</v>
       </c>
@@ -4097,7 +4105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="271" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A271" s="3" t="s">
         <v>270</v>
       </c>
@@ -4116,7 +4124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="273" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A273" s="3" t="s">
         <v>272</v>
       </c>
@@ -4124,7 +4132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="274" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A274" s="3" t="s">
         <v>273</v>
       </c>
@@ -4132,7 +4140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="275" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A275" s="3" t="s">
         <v>274</v>
       </c>
@@ -4140,7 +4148,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="276" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A276" s="15" t="s">
         <v>275</v>
       </c>
@@ -4184,7 +4192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="280" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A280" s="8" t="s">
         <v>279</v>
       </c>
@@ -4195,7 +4203,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="281" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A281" s="3" t="s">
         <v>280</v>
       </c>
@@ -4214,7 +4222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="283" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A283" s="3" t="s">
         <v>282</v>
       </c>
@@ -4222,7 +4230,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="284" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A284" s="3" t="s">
         <v>283</v>
       </c>
@@ -4233,7 +4241,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="285" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A285" s="3" t="s">
         <v>284</v>
       </c>
@@ -4241,7 +4249,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="286" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A286" s="3" t="s">
         <v>285</v>
       </c>
@@ -4249,7 +4257,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="287" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A287" s="3" t="s">
         <v>286</v>
       </c>
@@ -4257,7 +4265,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="288" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A288" s="3" t="s">
         <v>287</v>
       </c>
@@ -4276,7 +4284,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A290" s="3" t="s">
         <v>289</v>
       </c>
@@ -4284,7 +4292,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="291" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A291" s="3" t="s">
         <v>290</v>
       </c>
@@ -4292,7 +4300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="292" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A292" s="8" t="s">
         <v>291</v>
       </c>
@@ -4303,7 +4311,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="293" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A293" s="3" t="s">
         <v>292</v>
       </c>
@@ -4311,7 +4319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A294" s="3" t="s">
         <v>293</v>
       </c>
@@ -4322,7 +4330,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="295" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A295" s="3" t="s">
         <v>294</v>
       </c>
@@ -4330,7 +4338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A296" s="3" t="s">
         <v>295</v>
       </c>
@@ -4338,7 +4346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A297" s="3" t="s">
         <v>296</v>
       </c>
@@ -4346,7 +4354,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A298" s="3" t="s">
         <v>297</v>
       </c>
@@ -4365,7 +4373,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A300" s="16" t="s">
         <v>299</v>
       </c>
@@ -4373,7 +4381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A301" s="3" t="s">
         <v>300</v>
       </c>
@@ -4381,7 +4389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A302" s="15" t="s">
         <v>301</v>
       </c>
@@ -4392,7 +4400,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="303" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A303" s="8" t="s">
         <v>302</v>
       </c>
@@ -4403,7 +4411,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="304" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A304" s="17" t="s">
         <v>303</v>
       </c>
@@ -4411,7 +4419,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A305" s="3" t="s">
         <v>304</v>
       </c>
@@ -4419,7 +4427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A306" s="3" t="s">
         <v>305</v>
       </c>
@@ -4430,7 +4438,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="307" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A307" s="8" t="s">
         <v>306</v>
       </c>
@@ -4441,7 +4449,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="308" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A308" s="3" t="s">
         <v>307</v>
       </c>
@@ -4449,7 +4457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A309" s="3" t="s">
         <v>308</v>
       </c>
@@ -4457,7 +4465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="310" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A310" s="16" t="s">
         <v>309</v>
       </c>
@@ -4465,7 +4473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="311" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A311" s="3" t="s">
         <v>310</v>
       </c>
@@ -4473,7 +4481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="312" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A312" s="14" t="s">
         <v>311</v>
       </c>
@@ -4481,7 +4489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A313" s="20" t="s">
         <v>312</v>
       </c>
@@ -4492,7 +4500,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="314" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A314" s="3" t="s">
         <v>313</v>
       </c>
@@ -4500,7 +4508,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A315" s="3" t="s">
         <v>314</v>
       </c>
@@ -4521,14 +4529,8 @@
       <c r="C318" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C315" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="nucleus"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add more new script
</commit_message>
<xml_diff>
--- a/data/all_component_manual_check.xlsx
+++ b/data/all_component_manual_check.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA55A71-B895-A64D-9C30-6414F45668A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF4D514D-CB67-6244-AFFC-298F2D5DF4E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31960" yWindow="4580" windowWidth="26760" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="26880" windowHeight="15220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4540,6 +4540,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="23.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>